<commit_message>
agregamos función para buscar por nombre
hice una función para permitir buscar por nombre y la agregue a la opción 2 del menú
</commit_message>
<xml_diff>
--- a/proveedores_murmat.xlsx
+++ b/proveedores_murmat.xlsx
@@ -283,7 +283,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.5234375" defaultRowHeight="12.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <sheetData>
     <row r="1" ht="12.75" customHeight="1" s="3">
@@ -556,51 +556,6 @@
       <c r="G10" s="4" t="n"/>
       <c r="H10" s="4" t="n"/>
       <c r="I10" s="4" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>Pepito</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>01234567891</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>Ladrillos refractarios</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>Pepito gonzalez</t>
-        </is>
-      </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>conzales@gmail.com</t>
-        </is>
-      </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>42536457</t>
-        </is>
-      </c>
-      <c r="H11" s="4" t="inlineStr">
-        <is>
-          <t>inactivo</t>
-        </is>
-      </c>
-      <c r="I11" s="4" t="inlineStr">
-        <is>
-          <t>01/06/2026</t>
-        </is>
-      </c>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
Mejoras en el código
-Todos los Cuit con iones.
-Los cuit o nombres no se pueden repetir.
- cambio de la palara "salir" por "cancelar" (como en telegram)
-def reordenar id en el excel
</commit_message>
<xml_diff>
--- a/proveedores_murmat.xlsx
+++ b/proveedores_murmat.xlsx
@@ -283,7 +283,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.5234375" defaultRowHeight="12.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <sheetData>
     <row r="1" ht="12.75" customHeight="1" s="3">
@@ -334,203 +334,145 @@
       </c>
     </row>
     <row r="2" ht="12.75" customHeight="1" s="3">
-      <c r="A2" s="4" t="n">
+      <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Ceramicasdelsur</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>30-12345678-1</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Materias primas (Caolin-Tinkar)</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Ruiz Anastacio</t>
         </is>
       </c>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Ruizventas@galvacero.comceramicasdelsur</t>
         </is>
       </c>
-      <c r="G2" s="4" t="n">
+      <c r="G2" t="n">
         <v>42245678</v>
       </c>
-      <c r="H2" s="4" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Activo</t>
         </is>
       </c>
-      <c r="I2" s="4" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>06-2016</t>
         </is>
       </c>
     </row>
     <row r="3" ht="12.75" customHeight="1" s="3">
-      <c r="A3" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
         <is>
           <t>Edelflex</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>30124956341</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>Oxidos Y Carbonatos</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>Amparo Teodorico</t>
-        </is>
-      </c>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>Edelflexventas@edelflex.com.ar</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>42247898</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>Activo</t>
-        </is>
-      </c>
-      <c r="I3" s="4" t="inlineStr">
-        <is>
-          <t>10-06-2019</t>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>30-12495634-1</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Ceramicos Exterior</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Franco Dea</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>edelflex@gmail.com</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2956874632</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>12/06/2026</t>
         </is>
       </c>
     </row>
     <row r="4" ht="12.75" customHeight="1" s="3">
-      <c r="A4" s="4" t="n"/>
-      <c r="B4" s="4" t="n"/>
-      <c r="C4" s="4" t="n"/>
-      <c r="D4" s="4" t="n"/>
-      <c r="E4" s="4" t="n"/>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>mailto:Edelflexventas@edelflex.com.ar</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="n"/>
-      <c r="H4" s="4" t="n"/>
-      <c r="I4" s="4" t="n"/>
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Fart Construcciones</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>30-34297367-2</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Construccion Gral</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Mario Lauri</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>fartconstrucciones@gmail.com</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>3455987654</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>activo</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>12/06/2026</t>
+        </is>
+      </c>
     </row>
-    <row r="5" ht="12.75" customHeight="1" s="3">
-      <c r="A5" s="4" t="n"/>
-      <c r="B5" s="4" t="n"/>
-      <c r="C5" s="4" t="n"/>
-      <c r="D5" s="4" t="n"/>
-      <c r="E5" s="4" t="n"/>
-      <c r="F5" s="4" t="n"/>
-      <c r="G5" s="4" t="n"/>
-      <c r="H5" s="4" t="n"/>
-      <c r="I5" s="4" t="n"/>
-    </row>
-    <row r="6" ht="12.75" customHeight="1" s="3">
-      <c r="A6" s="4" t="n"/>
-      <c r="B6" s="4" t="n"/>
-      <c r="C6" s="4" t="n"/>
-      <c r="D6" s="4" t="n"/>
-      <c r="E6" s="4" t="n"/>
-      <c r="F6" s="4" t="n"/>
-      <c r="G6" s="4" t="n"/>
-      <c r="H6" s="4" t="n"/>
-      <c r="I6" s="4" t="n"/>
-    </row>
-    <row r="7" ht="12.75" customHeight="1" s="3">
-      <c r="A7" s="4" t="n"/>
-      <c r="B7" s="4" t="n"/>
-      <c r="C7" s="4" t="n"/>
-      <c r="D7" s="4" t="n"/>
-      <c r="E7" s="4" t="n"/>
-      <c r="F7" s="4" t="n"/>
-      <c r="G7" s="4" t="n"/>
-      <c r="H7" s="4" t="n"/>
-      <c r="I7" s="4" t="n"/>
-    </row>
-    <row r="8" ht="12.75" customHeight="1" s="3">
-      <c r="A8" s="4" t="n"/>
-      <c r="B8" s="4" t="n"/>
-      <c r="C8" s="4" t="n"/>
-      <c r="D8" s="4" t="n"/>
-      <c r="E8" s="4" t="n"/>
-      <c r="F8" s="4" t="n"/>
-      <c r="G8" s="4" t="n"/>
-      <c r="H8" s="4" t="n"/>
-      <c r="I8" s="4" t="n"/>
-    </row>
-    <row r="9" ht="12.75" customHeight="1" s="3">
-      <c r="A9" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>Frs Ceramicas</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>30124956341</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>Ceramicos Exterior</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>Franco Dea</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>ceramicas.frs@gmail.com</t>
-        </is>
-      </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>2944639875</t>
-        </is>
-      </c>
-      <c r="H9" s="4" t="inlineStr">
-        <is>
-          <t>activo</t>
-        </is>
-      </c>
-      <c r="I9" s="4" t="inlineStr">
-        <is>
-          <t>11/06/2026</t>
-        </is>
-      </c>
-    </row>
+    <row r="5" ht="12.75" customHeight="1" s="3"/>
+    <row r="6" ht="12.75" customHeight="1" s="3"/>
+    <row r="7" ht="12.75" customHeight="1" s="3"/>
+    <row r="8" ht="12.75" customHeight="1" s="3"/>
+    <row r="9" ht="12.75" customHeight="1" s="3"/>
     <row r="10" ht="12.75" customHeight="1" s="3"/>
   </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" display="Ruizventas@galvacero.comceramicasdelsur" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" display="Edelflexventas@edelflex.com.ar" r:id="rId2"/>
-  </hyperlinks>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" firstPageNumber="1" useFirstPageNumber="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
Nuevos cambios al código
-no repetir cuit ni nombre
- reordenar los id luego de una baja.
-camio palabra "salir" por "Cancelar"
-todos los CUIT se escriben con iones (-)
</commit_message>
<xml_diff>
--- a/proveedores_murmat.xlsx
+++ b/proveedores_murmat.xlsx
@@ -283,7 +283,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.5234375" defaultRowHeight="12.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <sheetData>
     <row r="1" ht="12.75" customHeight="1" s="3">
@@ -334,145 +334,203 @@
       </c>
     </row>
     <row r="2" ht="12.75" customHeight="1" s="3">
-      <c r="A2" t="n">
+      <c r="A2" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>Ceramicasdelsur</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>30-12345678-1</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>Materias primas (Caolin-Tinkar)</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>Ruiz Anastacio</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="5" t="inlineStr">
         <is>
           <t>Ruizventas@galvacero.comceramicasdelsur</t>
         </is>
       </c>
-      <c r="G2" t="n">
+      <c r="G2" s="4" t="n">
         <v>42245678</v>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" s="4" t="inlineStr">
         <is>
           <t>Activo</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" s="4" t="inlineStr">
         <is>
           <t>06-2016</t>
         </is>
       </c>
     </row>
     <row r="3" ht="12.75" customHeight="1" s="3">
-      <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="inlineStr">
+      <c r="A3" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Edelflex</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>30-12495634-1</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>30124956341</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Oxidos Y Carbonatos</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Amparo Teodorico</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Edelflexventas@edelflex.com.ar</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>42247898</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>10-06-2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="12.75" customHeight="1" s="3">
+      <c r="A4" s="4" t="n"/>
+      <c r="B4" s="4" t="n"/>
+      <c r="C4" s="4" t="n"/>
+      <c r="D4" s="4" t="n"/>
+      <c r="E4" s="4" t="n"/>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>mailto:Edelflexventas@edelflex.com.ar</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="n"/>
+      <c r="H4" s="4" t="n"/>
+      <c r="I4" s="4" t="n"/>
+    </row>
+    <row r="5" ht="12.75" customHeight="1" s="3">
+      <c r="A5" s="4" t="n"/>
+      <c r="B5" s="4" t="n"/>
+      <c r="C5" s="4" t="n"/>
+      <c r="D5" s="4" t="n"/>
+      <c r="E5" s="4" t="n"/>
+      <c r="F5" s="4" t="n"/>
+      <c r="G5" s="4" t="n"/>
+      <c r="H5" s="4" t="n"/>
+      <c r="I5" s="4" t="n"/>
+    </row>
+    <row r="6" ht="12.75" customHeight="1" s="3">
+      <c r="A6" s="4" t="n"/>
+      <c r="B6" s="4" t="n"/>
+      <c r="C6" s="4" t="n"/>
+      <c r="D6" s="4" t="n"/>
+      <c r="E6" s="4" t="n"/>
+      <c r="F6" s="4" t="n"/>
+      <c r="G6" s="4" t="n"/>
+      <c r="H6" s="4" t="n"/>
+      <c r="I6" s="4" t="n"/>
+    </row>
+    <row r="7" ht="12.75" customHeight="1" s="3">
+      <c r="A7" s="4" t="n"/>
+      <c r="B7" s="4" t="n"/>
+      <c r="C7" s="4" t="n"/>
+      <c r="D7" s="4" t="n"/>
+      <c r="E7" s="4" t="n"/>
+      <c r="F7" s="4" t="n"/>
+      <c r="G7" s="4" t="n"/>
+      <c r="H7" s="4" t="n"/>
+      <c r="I7" s="4" t="n"/>
+    </row>
+    <row r="8" ht="12.75" customHeight="1" s="3">
+      <c r="A8" s="4" t="n"/>
+      <c r="B8" s="4" t="n"/>
+      <c r="C8" s="4" t="n"/>
+      <c r="D8" s="4" t="n"/>
+      <c r="E8" s="4" t="n"/>
+      <c r="F8" s="4" t="n"/>
+      <c r="G8" s="4" t="n"/>
+      <c r="H8" s="4" t="n"/>
+      <c r="I8" s="4" t="n"/>
+    </row>
+    <row r="9" ht="12.75" customHeight="1" s="3">
+      <c r="A9" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Frs Ceramicas</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>30124956341</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>Ceramicos Exterior</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>Franco Dea</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>edelflex@gmail.com</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>2956874632</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>ceramicas.frs@gmail.com</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>2944639875</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
         <is>
           <t>activo</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>12/06/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="12.75" customHeight="1" s="3">
-      <c r="A4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Fart Construcciones</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>30-34297367-2</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Construccion Gral</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Mario Lauri</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>fartconstrucciones@gmail.com</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>3455987654</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>activo</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>12/06/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="12.75" customHeight="1" s="3"/>
-    <row r="6" ht="12.75" customHeight="1" s="3"/>
-    <row r="7" ht="12.75" customHeight="1" s="3"/>
-    <row r="8" ht="12.75" customHeight="1" s="3"/>
-    <row r="9" ht="12.75" customHeight="1" s="3"/>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>11/06/2026</t>
+        </is>
+      </c>
+    </row>
     <row r="10" ht="12.75" customHeight="1" s="3"/>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" display="Ruizventas@galvacero.comceramicasdelsur" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" display="Edelflexventas@edelflex.com.ar" r:id="rId2"/>
+  </hyperlinks>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" firstPageNumber="1" useFirstPageNumber="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>